<commit_message>
agregando funcionalidades y partidos
</commit_message>
<xml_diff>
--- a/creando_dataset_modificado.xlsx
+++ b/creando_dataset_modificado.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="181">
   <si>
     <t>Partido_id</t>
   </si>
@@ -555,6 +555,9 @@
   <si>
     <t>2025-10-22</t>
   </si>
+  <si>
+    <t>2025-11-4</t>
+  </si>
 </sst>
 </file>
 
@@ -571,7 +574,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -635,19 +638,19 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -961,152 +964,152 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:EJ52"/>
+  <dimension ref="A1:EJ60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="10" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="10" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="10" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="10" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="36" max="36" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="37" max="37" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="38" max="38" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="39" max="39" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="40" max="40" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="41" max="41" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="42" max="42" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="43" max="43" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="44" max="44" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="45" max="45" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="46" max="46" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="47" max="47" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="48" max="48" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="49" max="49" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="50" max="50" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="51" max="51" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="52" max="52" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="53" max="53" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="54" max="54" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="55" max="55" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="56" max="56" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="57" max="57" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="58" max="58" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="59" max="59" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="60" max="60" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="61" max="61" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="62" max="62" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="63" max="63" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="64" max="64" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="65" max="65" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="66" max="66" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="67" max="67" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="68" max="68" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="69" max="69" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="70" max="70" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="71" max="71" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="72" max="72" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="73" max="73" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="74" max="74" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="75" max="75" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="76" max="76" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="77" max="77" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="78" max="78" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="79" max="79" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="80" max="80" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="81" max="81" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="82" max="82" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="83" max="83" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="84" max="84" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="85" max="85" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="86" max="86" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="87" max="87" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="88" max="88" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="89" max="89" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="90" max="90" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="91" max="91" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="92" max="92" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="93" max="93" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="94" max="94" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="95" max="95" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="96" max="96" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="97" max="97" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="98" max="98" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="99" max="99" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="100" max="100" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="101" max="101" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="102" max="102" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="103" max="103" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="104" max="104" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="105" max="105" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="106" max="106" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="107" max="107" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="108" max="108" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="109" max="109" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="110" max="110" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="111" max="111" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="112" max="112" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="113" max="113" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="114" max="114" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="115" max="115" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="116" max="116" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="117" max="117" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="118" max="118" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="119" max="119" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="120" max="120" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="121" max="121" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="122" max="122" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="123" max="123" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="124" max="124" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="125" max="125" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="126" max="126" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="127" max="127" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="128" max="128" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="129" max="129" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="130" max="130" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="131" max="131" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="132" max="132" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="133" max="133" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="134" max="134" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="135" max="135" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="136" max="136" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="137" max="137" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="138" max="138" style="9" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="139" max="139" style="11" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="140" max="140" style="11" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="37" max="37" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="38" max="38" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="39" max="39" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="40" max="40" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="41" max="41" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="42" max="42" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="43" max="43" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="44" max="44" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="45" max="45" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="46" max="46" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="47" max="47" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="48" max="48" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="49" max="49" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="50" max="50" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="51" max="51" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="52" max="52" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="53" max="53" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="54" max="54" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="55" max="55" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="56" max="56" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="57" max="57" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="58" max="58" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="59" max="59" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="60" max="60" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="61" max="61" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="62" max="62" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="63" max="63" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="64" max="64" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="65" max="65" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="66" max="66" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="67" max="67" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="68" max="68" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="69" max="69" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="70" max="70" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="71" max="71" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="72" max="72" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="73" max="73" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="74" max="74" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="75" max="75" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="76" max="76" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="77" max="77" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="78" max="78" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="79" max="79" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="80" max="80" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="81" max="81" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="82" max="82" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="83" max="83" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="84" max="84" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="85" max="85" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="86" max="86" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="87" max="87" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="88" max="88" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="89" max="89" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="90" max="90" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="91" max="91" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="92" max="92" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="93" max="93" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="94" max="94" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="95" max="95" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="96" max="96" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="97" max="97" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="98" max="98" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="99" max="99" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="100" max="100" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="101" max="101" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="102" max="102" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="103" max="103" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="104" max="104" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="105" max="105" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="106" max="106" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="107" max="107" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="108" max="108" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="109" max="109" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="110" max="110" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="111" max="111" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="112" max="112" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="113" max="113" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="114" max="114" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="115" max="115" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="116" max="116" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="117" max="117" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="118" max="118" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="119" max="119" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="120" max="120" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="121" max="121" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="122" max="122" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="123" max="123" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="124" max="124" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="125" max="125" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="126" max="126" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="127" max="127" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="128" max="128" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="129" max="129" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="130" max="130" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="131" max="131" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="132" max="132" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="133" max="133" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="134" max="134" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="135" max="135" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="136" max="136" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="137" max="137" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="138" max="138" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="139" max="139" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="140" max="140" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7364,7 +7367,7 @@
       <c r="EI15" s="7"/>
       <c r="EJ15" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -7780,7 +7783,7 @@
       <c r="EI16" s="7"/>
       <c r="EJ16" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -8196,7 +8199,7 @@
       <c r="EI17" s="7"/>
       <c r="EJ17" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -8612,7 +8615,7 @@
       <c r="EI18" s="7"/>
       <c r="EJ18" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -9028,7 +9031,7 @@
       <c r="EI19" s="7"/>
       <c r="EJ19" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -9444,7 +9447,7 @@
       <c r="EI20" s="7"/>
       <c r="EJ20" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -9860,7 +9863,7 @@
       <c r="EI21" s="7"/>
       <c r="EJ21" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="4">
         <v>21</v>
       </c>
@@ -10276,7 +10279,7 @@
       <c r="EI22" s="7"/>
       <c r="EJ22" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="4">
         <v>22</v>
       </c>
@@ -10692,7 +10695,7 @@
       <c r="EI23" s="7"/>
       <c r="EJ23" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="4">
         <v>23</v>
       </c>
@@ -11108,7 +11111,7 @@
       <c r="EI24" s="7"/>
       <c r="EJ24" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="4">
         <v>24</v>
       </c>
@@ -11524,7 +11527,7 @@
       <c r="EI25" s="7"/>
       <c r="EJ25" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="4">
         <v>25</v>
       </c>
@@ -11940,7 +11943,7 @@
       <c r="EI26" s="7"/>
       <c r="EJ26" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -12356,7 +12359,7 @@
       <c r="EI27" s="7"/>
       <c r="EJ27" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="4">
         <v>27</v>
       </c>
@@ -12772,7 +12775,7 @@
       <c r="EI28" s="7"/>
       <c r="EJ28" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="4">
         <v>28</v>
       </c>
@@ -13186,7 +13189,7 @@
       <c r="EI29" s="7"/>
       <c r="EJ29" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -13602,7 +13605,7 @@
       <c r="EI30" s="7"/>
       <c r="EJ30" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="4">
         <v>30</v>
       </c>
@@ -14020,7 +14023,7 @@
       <c r="EI31" s="7"/>
       <c r="EJ31" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -14436,7 +14439,7 @@
       <c r="EI32" s="7"/>
       <c r="EJ32" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="4">
         <v>32</v>
       </c>
@@ -14854,7 +14857,7 @@
       <c r="EI33" s="7"/>
       <c r="EJ33" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="4">
         <v>33</v>
       </c>
@@ -15272,7 +15275,7 @@
       <c r="EI34" s="7"/>
       <c r="EJ34" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="4">
         <v>34</v>
       </c>
@@ -15690,7 +15693,7 @@
       <c r="EI35" s="7"/>
       <c r="EJ35" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="4">
         <v>35</v>
       </c>
@@ -16108,7 +16111,7 @@
       <c r="EI36" s="7"/>
       <c r="EJ36" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="4">
         <v>36</v>
       </c>
@@ -16526,7 +16529,7 @@
       <c r="EI37" s="7"/>
       <c r="EJ37" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="4">
         <v>37</v>
       </c>
@@ -16944,7 +16947,7 @@
       <c r="EI38" s="7"/>
       <c r="EJ38" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
       <c r="A39" s="4">
         <v>38</v>
       </c>
@@ -17362,7 +17365,7 @@
       <c r="EI39" s="7"/>
       <c r="EJ39" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
       <c r="A40" s="4">
         <v>39</v>
       </c>
@@ -17780,7 +17783,7 @@
       <c r="EI40" s="7"/>
       <c r="EJ40" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
       <c r="A41" s="4">
         <v>40</v>
       </c>
@@ -18198,7 +18201,7 @@
       <c r="EI41" s="7"/>
       <c r="EJ41" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
       <c r="A42" s="4">
         <v>41</v>
       </c>
@@ -18616,7 +18619,7 @@
       <c r="EI42" s="7"/>
       <c r="EJ42" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
       <c r="A43" s="4">
         <v>42</v>
       </c>
@@ -19034,7 +19037,7 @@
       <c r="EI43" s="7"/>
       <c r="EJ43" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
       <c r="A44" s="4">
         <v>43</v>
       </c>
@@ -19452,7 +19455,7 @@
       <c r="EI44" s="7"/>
       <c r="EJ44" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
       <c r="A45" s="4">
         <v>44</v>
       </c>
@@ -19870,7 +19873,7 @@
       <c r="EI45" s="7"/>
       <c r="EJ45" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
       <c r="A46" s="4">
         <v>45</v>
       </c>
@@ -20288,7 +20291,7 @@
       <c r="EI46" s="7"/>
       <c r="EJ46" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
       <c r="A47" s="4">
         <v>46</v>
       </c>
@@ -20706,7 +20709,7 @@
       <c r="EI47" s="7"/>
       <c r="EJ47" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
       <c r="A48" s="4">
         <v>47</v>
       </c>
@@ -21124,7 +21127,7 @@
       <c r="EI48" s="7"/>
       <c r="EJ48" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
       <c r="A49" s="4">
         <v>48</v>
       </c>
@@ -21542,7 +21545,7 @@
       <c r="EI49" s="7"/>
       <c r="EJ49" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
       <c r="A50" s="4">
         <v>49</v>
       </c>
@@ -21960,7 +21963,7 @@
       <c r="EI50" s="7"/>
       <c r="EJ50" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
       <c r="A51" s="4">
         <v>50</v>
       </c>
@@ -22378,7 +22381,7 @@
       <c r="EI51" s="7"/>
       <c r="EJ51" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
       <c r="A52" s="4">
         <v>51</v>
       </c>
@@ -22795,6 +22798,3350 @@
       </c>
       <c r="EI52" s="7"/>
       <c r="EJ52" s="7"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
+      <c r="A53" s="4">
+        <v>52</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="E53" s="4">
+        <v>1</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="G53" s="4">
+        <v>1</v>
+      </c>
+      <c r="H53" s="4">
+        <v>0</v>
+      </c>
+      <c r="I53" s="4">
+        <v>1</v>
+      </c>
+      <c r="J53" s="4">
+        <v>0</v>
+      </c>
+      <c r="K53" s="4">
+        <v>27</v>
+      </c>
+      <c r="L53" s="4">
+        <v>9</v>
+      </c>
+      <c r="M53" s="4">
+        <v>6</v>
+      </c>
+      <c r="N53" s="4">
+        <v>12</v>
+      </c>
+      <c r="O53" s="4">
+        <v>1</v>
+      </c>
+      <c r="P53" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="4">
+        <v>1</v>
+      </c>
+      <c r="R53" s="4">
+        <v>3</v>
+      </c>
+      <c r="S53" s="4">
+        <v>0</v>
+      </c>
+      <c r="T53" s="4">
+        <v>1</v>
+      </c>
+      <c r="U53" s="4">
+        <v>0</v>
+      </c>
+      <c r="V53" s="4">
+        <v>0</v>
+      </c>
+      <c r="W53" s="4">
+        <v>0</v>
+      </c>
+      <c r="X53" s="4">
+        <v>82</v>
+      </c>
+      <c r="Y53" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z53" s="4">
+        <v>13</v>
+      </c>
+      <c r="AA53" s="4">
+        <v>1</v>
+      </c>
+      <c r="AB53" s="4">
+        <v>16</v>
+      </c>
+      <c r="AC53" s="4">
+        <v>15</v>
+      </c>
+      <c r="AD53" s="4">
+        <v>21</v>
+      </c>
+      <c r="AE53" s="4">
+        <v>12</v>
+      </c>
+      <c r="AF53" s="4">
+        <v>62</v>
+      </c>
+      <c r="AG53" s="4">
+        <v>91</v>
+      </c>
+      <c r="AH53" s="4">
+        <v>558</v>
+      </c>
+      <c r="AI53" s="4">
+        <v>614</v>
+      </c>
+      <c r="AJ53" s="4">
+        <v>161</v>
+      </c>
+      <c r="AK53" s="4">
+        <v>353</v>
+      </c>
+      <c r="AL53" s="4">
+        <v>44</v>
+      </c>
+      <c r="AM53" s="4">
+        <v>98</v>
+      </c>
+      <c r="AN53" s="4">
+        <v>170</v>
+      </c>
+      <c r="AO53" s="4">
+        <v>147</v>
+      </c>
+      <c r="AP53" s="4">
+        <v>21</v>
+      </c>
+      <c r="AQ53" s="4">
+        <v>77</v>
+      </c>
+      <c r="AR53" s="4">
+        <v>66</v>
+      </c>
+      <c r="AS53" s="4">
+        <v>19</v>
+      </c>
+      <c r="AT53" s="4">
+        <v>32</v>
+      </c>
+      <c r="AU53" s="4">
+        <v>6</v>
+      </c>
+      <c r="AV53" s="4">
+        <v>19</v>
+      </c>
+      <c r="AW53" s="4">
+        <v>190</v>
+      </c>
+      <c r="AX53" s="4">
+        <v>27</v>
+      </c>
+      <c r="AY53" s="4">
+        <v>5</v>
+      </c>
+      <c r="AZ53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BA53" s="4">
+        <v>23</v>
+      </c>
+      <c r="BB53" s="4">
+        <v>9</v>
+      </c>
+      <c r="BC53" s="4">
+        <v>14</v>
+      </c>
+      <c r="BD53" s="4">
+        <v>11</v>
+      </c>
+      <c r="BE53" s="4">
+        <v>16</v>
+      </c>
+      <c r="BF53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BG53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BH53" s="4">
+        <v>1</v>
+      </c>
+      <c r="BI53" s="4">
+        <v>6</v>
+      </c>
+      <c r="BJ53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BK53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BL53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BM53" s="4">
+        <v>2</v>
+      </c>
+      <c r="BN53" s="4">
+        <v>1</v>
+      </c>
+      <c r="BO53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ53" s="4">
+        <v>1</v>
+      </c>
+      <c r="BR53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS53" s="4">
+        <v>10</v>
+      </c>
+      <c r="BT53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU53" s="4">
+        <v>1</v>
+      </c>
+      <c r="BV53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BW53" s="4">
+        <v>0</v>
+      </c>
+      <c r="BX53" s="4">
+        <v>12</v>
+      </c>
+      <c r="BY53" s="4">
+        <v>6</v>
+      </c>
+      <c r="BZ53" s="4">
+        <v>1</v>
+      </c>
+      <c r="CA53" s="4">
+        <v>5</v>
+      </c>
+      <c r="CB53" s="4">
+        <v>0</v>
+      </c>
+      <c r="CC53" s="4">
+        <v>0</v>
+      </c>
+      <c r="CD53" s="4">
+        <v>0</v>
+      </c>
+      <c r="CE53" s="4">
+        <v>5</v>
+      </c>
+      <c r="CF53" s="4">
+        <v>1</v>
+      </c>
+      <c r="CG53" s="4">
+        <v>0</v>
+      </c>
+      <c r="CH53" s="4">
+        <v>0</v>
+      </c>
+      <c r="CI53" s="4">
+        <v>0</v>
+      </c>
+      <c r="CJ53" s="4">
+        <v>0</v>
+      </c>
+      <c r="CK53" s="4">
+        <v>32</v>
+      </c>
+      <c r="CL53" s="4">
+        <v>1</v>
+      </c>
+      <c r="CM53" s="4">
+        <v>7</v>
+      </c>
+      <c r="CN53" s="4">
+        <v>2</v>
+      </c>
+      <c r="CO53" s="4">
+        <v>13</v>
+      </c>
+      <c r="CP53" s="4">
+        <v>7</v>
+      </c>
+      <c r="CQ53" s="4">
+        <v>8</v>
+      </c>
+      <c r="CR53" s="4">
+        <v>6</v>
+      </c>
+      <c r="CS53" s="4">
+        <v>38</v>
+      </c>
+      <c r="CT53" s="4">
+        <v>84</v>
+      </c>
+      <c r="CU53" s="4">
+        <v>270</v>
+      </c>
+      <c r="CV53" s="4">
+        <v>322</v>
+      </c>
+      <c r="CW53" s="4">
+        <v>94</v>
+      </c>
+      <c r="CX53" s="4">
+        <v>151</v>
+      </c>
+      <c r="CY53" s="4">
+        <v>25</v>
+      </c>
+      <c r="CZ53" s="4">
+        <v>55</v>
+      </c>
+      <c r="DA53" s="4">
+        <v>74</v>
+      </c>
+      <c r="DB53" s="4">
+        <v>65</v>
+      </c>
+      <c r="DC53" s="4">
+        <v>10</v>
+      </c>
+      <c r="DD53" s="4">
+        <v>23</v>
+      </c>
+      <c r="DE53" s="4">
+        <v>16</v>
+      </c>
+      <c r="DF53" s="4">
+        <v>5</v>
+      </c>
+      <c r="DG53" s="4">
+        <v>6</v>
+      </c>
+      <c r="DH53" s="4">
+        <v>1</v>
+      </c>
+      <c r="DI53" s="4">
+        <v>18</v>
+      </c>
+      <c r="DJ53" s="4">
+        <v>186</v>
+      </c>
+      <c r="DK53" s="4">
+        <v>29</v>
+      </c>
+      <c r="DL53" s="4">
+        <v>12</v>
+      </c>
+      <c r="DM53" s="4">
+        <v>0</v>
+      </c>
+      <c r="DN53" s="4">
+        <v>15</v>
+      </c>
+      <c r="DO53" s="4">
+        <v>4</v>
+      </c>
+      <c r="DP53" s="4">
+        <v>11</v>
+      </c>
+      <c r="DQ53" s="4">
+        <v>14</v>
+      </c>
+      <c r="DR53" s="4">
+        <v>18</v>
+      </c>
+      <c r="DS53" s="4">
+        <v>1</v>
+      </c>
+      <c r="DT53" s="4">
+        <v>0</v>
+      </c>
+      <c r="DU53" s="4">
+        <v>0</v>
+      </c>
+      <c r="DV53" s="4">
+        <v>8</v>
+      </c>
+      <c r="DW53" s="4">
+        <v>0</v>
+      </c>
+      <c r="DX53" s="4">
+        <v>0</v>
+      </c>
+      <c r="DY53" s="4">
+        <v>0</v>
+      </c>
+      <c r="DZ53" s="4">
+        <v>1</v>
+      </c>
+      <c r="EA53" s="4">
+        <v>0</v>
+      </c>
+      <c r="EB53" s="4">
+        <v>0</v>
+      </c>
+      <c r="EC53" s="4">
+        <v>0</v>
+      </c>
+      <c r="ED53" s="4">
+        <v>0</v>
+      </c>
+      <c r="EE53" s="4">
+        <v>0</v>
+      </c>
+      <c r="EF53" s="4">
+        <v>18</v>
+      </c>
+      <c r="EG53" s="4">
+        <v>2</v>
+      </c>
+      <c r="EH53" s="4">
+        <v>8</v>
+      </c>
+      <c r="EI53" s="7"/>
+      <c r="EJ53" s="7"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
+      <c r="A54" s="4">
+        <v>53</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="E54" s="4">
+        <v>1</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="G54" s="4">
+        <v>4</v>
+      </c>
+      <c r="H54" s="4">
+        <v>0</v>
+      </c>
+      <c r="I54" s="4">
+        <v>3</v>
+      </c>
+      <c r="J54" s="4">
+        <v>1</v>
+      </c>
+      <c r="K54" s="4">
+        <v>27</v>
+      </c>
+      <c r="L54" s="4">
+        <v>11</v>
+      </c>
+      <c r="M54" s="4">
+        <v>7</v>
+      </c>
+      <c r="N54" s="4">
+        <v>9</v>
+      </c>
+      <c r="O54" s="4">
+        <v>1</v>
+      </c>
+      <c r="P54" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="4">
+        <v>1</v>
+      </c>
+      <c r="R54" s="4">
+        <v>4</v>
+      </c>
+      <c r="S54" s="4">
+        <v>2</v>
+      </c>
+      <c r="T54" s="4">
+        <v>2</v>
+      </c>
+      <c r="U54" s="4">
+        <v>0</v>
+      </c>
+      <c r="V54" s="4">
+        <v>0</v>
+      </c>
+      <c r="W54" s="4">
+        <v>0</v>
+      </c>
+      <c r="X54" s="4">
+        <v>81</v>
+      </c>
+      <c r="Y54" s="4">
+        <v>3</v>
+      </c>
+      <c r="Z54" s="4">
+        <v>9</v>
+      </c>
+      <c r="AA54" s="4">
+        <v>1</v>
+      </c>
+      <c r="AB54" s="4">
+        <v>20</v>
+      </c>
+      <c r="AC54" s="4">
+        <v>15</v>
+      </c>
+      <c r="AD54" s="4">
+        <v>23</v>
+      </c>
+      <c r="AE54" s="4">
+        <v>21</v>
+      </c>
+      <c r="AF54" s="4">
+        <v>59</v>
+      </c>
+      <c r="AG54" s="4">
+        <v>92</v>
+      </c>
+      <c r="AH54" s="4">
+        <v>680</v>
+      </c>
+      <c r="AI54" s="4">
+        <v>737</v>
+      </c>
+      <c r="AJ54" s="4">
+        <v>171</v>
+      </c>
+      <c r="AK54" s="4">
+        <v>461</v>
+      </c>
+      <c r="AL54" s="4">
+        <v>48</v>
+      </c>
+      <c r="AM54" s="4">
+        <v>134</v>
+      </c>
+      <c r="AN54" s="4">
+        <v>176</v>
+      </c>
+      <c r="AO54" s="4">
+        <v>185</v>
+      </c>
+      <c r="AP54" s="4">
+        <v>3</v>
+      </c>
+      <c r="AQ54" s="4">
+        <v>74</v>
+      </c>
+      <c r="AR54" s="4">
+        <v>60</v>
+      </c>
+      <c r="AS54" s="4">
+        <v>18</v>
+      </c>
+      <c r="AT54" s="4">
+        <v>6</v>
+      </c>
+      <c r="AU54" s="4">
+        <v>1</v>
+      </c>
+      <c r="AV54" s="4">
+        <v>16</v>
+      </c>
+      <c r="AW54" s="4">
+        <v>157</v>
+      </c>
+      <c r="AX54" s="4">
+        <v>38</v>
+      </c>
+      <c r="AY54" s="4">
+        <v>1</v>
+      </c>
+      <c r="AZ54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BA54" s="4">
+        <v>15</v>
+      </c>
+      <c r="BB54" s="4">
+        <v>5</v>
+      </c>
+      <c r="BC54" s="4">
+        <v>10</v>
+      </c>
+      <c r="BD54" s="4">
+        <v>9</v>
+      </c>
+      <c r="BE54" s="4">
+        <v>9</v>
+      </c>
+      <c r="BF54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BG54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BH54" s="4">
+        <v>1</v>
+      </c>
+      <c r="BI54" s="4">
+        <v>2</v>
+      </c>
+      <c r="BJ54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BK54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BL54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BM54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BN54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BO54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ54" s="4">
+        <v>1</v>
+      </c>
+      <c r="BR54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS54" s="4">
+        <v>14</v>
+      </c>
+      <c r="BT54" s="4">
+        <v>2</v>
+      </c>
+      <c r="BU54" s="4">
+        <v>6</v>
+      </c>
+      <c r="BV54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BW54" s="4">
+        <v>0</v>
+      </c>
+      <c r="BX54" s="4">
+        <v>5</v>
+      </c>
+      <c r="BY54" s="4">
+        <v>2</v>
+      </c>
+      <c r="BZ54" s="4">
+        <v>2</v>
+      </c>
+      <c r="CA54" s="4">
+        <v>1</v>
+      </c>
+      <c r="CB54" s="4">
+        <v>0</v>
+      </c>
+      <c r="CC54" s="4">
+        <v>0</v>
+      </c>
+      <c r="CD54" s="4">
+        <v>0</v>
+      </c>
+      <c r="CE54" s="4">
+        <v>1</v>
+      </c>
+      <c r="CF54" s="4">
+        <v>0</v>
+      </c>
+      <c r="CG54" s="4">
+        <v>0</v>
+      </c>
+      <c r="CH54" s="4">
+        <v>0</v>
+      </c>
+      <c r="CI54" s="4">
+        <v>0</v>
+      </c>
+      <c r="CJ54" s="4">
+        <v>0</v>
+      </c>
+      <c r="CK54" s="4">
+        <v>27</v>
+      </c>
+      <c r="CL54" s="4">
+        <v>0</v>
+      </c>
+      <c r="CM54" s="4">
+        <v>1</v>
+      </c>
+      <c r="CN54" s="4">
+        <v>0</v>
+      </c>
+      <c r="CO54" s="4">
+        <v>16</v>
+      </c>
+      <c r="CP54" s="4">
+        <v>7</v>
+      </c>
+      <c r="CQ54" s="4">
+        <v>4</v>
+      </c>
+      <c r="CR54" s="4">
+        <v>1</v>
+      </c>
+      <c r="CS54" s="4">
+        <v>41</v>
+      </c>
+      <c r="CT54" s="4">
+        <v>88</v>
+      </c>
+      <c r="CU54" s="4">
+        <v>367</v>
+      </c>
+      <c r="CV54" s="4">
+        <v>419</v>
+      </c>
+      <c r="CW54" s="4">
+        <v>75</v>
+      </c>
+      <c r="CX54" s="4">
+        <v>252</v>
+      </c>
+      <c r="CY54" s="4">
+        <v>40</v>
+      </c>
+      <c r="CZ54" s="4">
+        <v>85</v>
+      </c>
+      <c r="DA54" s="4">
+        <v>82</v>
+      </c>
+      <c r="DB54" s="4">
+        <v>82</v>
+      </c>
+      <c r="DC54" s="4">
+        <v>15</v>
+      </c>
+      <c r="DD54" s="4">
+        <v>33</v>
+      </c>
+      <c r="DE54" s="4">
+        <v>20</v>
+      </c>
+      <c r="DF54" s="4">
+        <v>5</v>
+      </c>
+      <c r="DG54" s="4">
+        <v>43</v>
+      </c>
+      <c r="DH54" s="4">
+        <v>3</v>
+      </c>
+      <c r="DI54" s="4">
+        <v>7</v>
+      </c>
+      <c r="DJ54" s="4">
+        <v>160</v>
+      </c>
+      <c r="DK54" s="4">
+        <v>27</v>
+      </c>
+      <c r="DL54" s="4">
+        <v>9</v>
+      </c>
+      <c r="DM54" s="4">
+        <v>0</v>
+      </c>
+      <c r="DN54" s="4">
+        <v>15</v>
+      </c>
+      <c r="DO54" s="4">
+        <v>6</v>
+      </c>
+      <c r="DP54" s="4">
+        <v>9</v>
+      </c>
+      <c r="DQ54" s="4">
+        <v>23</v>
+      </c>
+      <c r="DR54" s="4">
+        <v>26</v>
+      </c>
+      <c r="DS54" s="4">
+        <v>4</v>
+      </c>
+      <c r="DT54" s="4">
+        <v>0</v>
+      </c>
+      <c r="DU54" s="4">
+        <v>0</v>
+      </c>
+      <c r="DV54" s="4">
+        <v>7</v>
+      </c>
+      <c r="DW54" s="4">
+        <v>0</v>
+      </c>
+      <c r="DX54" s="4">
+        <v>0</v>
+      </c>
+      <c r="DY54" s="4">
+        <v>0</v>
+      </c>
+      <c r="DZ54" s="4">
+        <v>3</v>
+      </c>
+      <c r="EA54" s="4">
+        <v>2</v>
+      </c>
+      <c r="EB54" s="4">
+        <v>1</v>
+      </c>
+      <c r="EC54" s="4">
+        <v>0</v>
+      </c>
+      <c r="ED54" s="4">
+        <v>0</v>
+      </c>
+      <c r="EE54" s="4">
+        <v>0</v>
+      </c>
+      <c r="EF54" s="4">
+        <v>3</v>
+      </c>
+      <c r="EG54" s="4">
+        <v>0</v>
+      </c>
+      <c r="EH54" s="4">
+        <v>0</v>
+      </c>
+      <c r="EI54" s="7"/>
+      <c r="EJ54" s="7"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
+      <c r="A55" s="4">
+        <v>54</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="E55" s="4">
+        <v>1</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="G55" s="4">
+        <v>0</v>
+      </c>
+      <c r="H55" s="4">
+        <v>0</v>
+      </c>
+      <c r="I55" s="4">
+        <v>0</v>
+      </c>
+      <c r="J55" s="4">
+        <v>0</v>
+      </c>
+      <c r="K55" s="4">
+        <v>18</v>
+      </c>
+      <c r="L55" s="4">
+        <v>2</v>
+      </c>
+      <c r="M55" s="4">
+        <v>8</v>
+      </c>
+      <c r="N55" s="4">
+        <v>8</v>
+      </c>
+      <c r="O55" s="4">
+        <v>0</v>
+      </c>
+      <c r="P55" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="4">
+        <v>0</v>
+      </c>
+      <c r="R55" s="4">
+        <v>0</v>
+      </c>
+      <c r="S55" s="4">
+        <v>3</v>
+      </c>
+      <c r="T55" s="4">
+        <v>0</v>
+      </c>
+      <c r="U55" s="4">
+        <v>0</v>
+      </c>
+      <c r="V55" s="4">
+        <v>0</v>
+      </c>
+      <c r="W55" s="4">
+        <v>0</v>
+      </c>
+      <c r="X55" s="4">
+        <v>69</v>
+      </c>
+      <c r="Y55" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z55" s="4">
+        <v>5</v>
+      </c>
+      <c r="AA55" s="4">
+        <v>1</v>
+      </c>
+      <c r="AB55" s="4">
+        <v>22</v>
+      </c>
+      <c r="AC55" s="4">
+        <v>19</v>
+      </c>
+      <c r="AD55" s="4">
+        <v>17</v>
+      </c>
+      <c r="AE55" s="4">
+        <v>4</v>
+      </c>
+      <c r="AF55" s="4">
+        <v>61</v>
+      </c>
+      <c r="AG55" s="4">
+        <v>90</v>
+      </c>
+      <c r="AH55" s="4">
+        <v>611</v>
+      </c>
+      <c r="AI55" s="4">
+        <v>682</v>
+      </c>
+      <c r="AJ55" s="4">
+        <v>201</v>
+      </c>
+      <c r="AK55" s="4">
+        <v>363</v>
+      </c>
+      <c r="AL55" s="4">
+        <v>47</v>
+      </c>
+      <c r="AM55" s="4">
+        <v>138</v>
+      </c>
+      <c r="AN55" s="4">
+        <v>122</v>
+      </c>
+      <c r="AO55" s="4">
+        <v>158</v>
+      </c>
+      <c r="AP55" s="4">
+        <v>10</v>
+      </c>
+      <c r="AQ55" s="4">
+        <v>73</v>
+      </c>
+      <c r="AR55" s="4">
+        <v>35</v>
+      </c>
+      <c r="AS55" s="4">
+        <v>11</v>
+      </c>
+      <c r="AT55" s="4">
+        <v>24</v>
+      </c>
+      <c r="AU55" s="4">
+        <v>6</v>
+      </c>
+      <c r="AV55" s="4">
+        <v>25</v>
+      </c>
+      <c r="AW55" s="4">
+        <v>189</v>
+      </c>
+      <c r="AX55" s="4">
+        <v>40</v>
+      </c>
+      <c r="AY55" s="4">
+        <v>2</v>
+      </c>
+      <c r="AZ55" s="4">
+        <v>0</v>
+      </c>
+      <c r="BA55" s="4">
+        <v>10</v>
+      </c>
+      <c r="BB55" s="4">
+        <v>5</v>
+      </c>
+      <c r="BC55" s="4">
+        <v>5</v>
+      </c>
+      <c r="BD55" s="4">
+        <v>12</v>
+      </c>
+      <c r="BE55" s="4">
+        <v>17</v>
+      </c>
+      <c r="BF55" s="4">
+        <v>0</v>
+      </c>
+      <c r="BG55" s="4">
+        <v>0</v>
+      </c>
+      <c r="BH55" s="4">
+        <v>1</v>
+      </c>
+      <c r="BI55" s="4">
+        <v>3</v>
+      </c>
+      <c r="BJ55" s="4">
+        <v>0</v>
+      </c>
+      <c r="BK55" s="4">
+        <v>0</v>
+      </c>
+      <c r="BL55" s="4">
+        <v>0</v>
+      </c>
+      <c r="BM55" s="4">
+        <v>1</v>
+      </c>
+      <c r="BN55" s="4">
+        <v>0</v>
+      </c>
+      <c r="BO55" s="4">
+        <v>1</v>
+      </c>
+      <c r="BP55" s="4">
+        <v>1</v>
+      </c>
+      <c r="BQ55" s="4">
+        <v>3</v>
+      </c>
+      <c r="BR55" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS55" s="4">
+        <v>12</v>
+      </c>
+      <c r="BT55" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU55" s="4">
+        <v>4</v>
+      </c>
+      <c r="BV55" s="4">
+        <v>0</v>
+      </c>
+      <c r="BW55" s="4">
+        <v>0</v>
+      </c>
+      <c r="BX55" s="4">
+        <v>7</v>
+      </c>
+      <c r="BY55" s="4">
+        <v>3</v>
+      </c>
+      <c r="BZ55" s="4">
+        <v>2</v>
+      </c>
+      <c r="CA55" s="4">
+        <v>2</v>
+      </c>
+      <c r="CB55" s="4">
+        <v>0</v>
+      </c>
+      <c r="CC55" s="4">
+        <v>0</v>
+      </c>
+      <c r="CD55" s="4">
+        <v>0</v>
+      </c>
+      <c r="CE55" s="4">
+        <v>2</v>
+      </c>
+      <c r="CF55" s="4">
+        <v>0</v>
+      </c>
+      <c r="CG55" s="4">
+        <v>0</v>
+      </c>
+      <c r="CH55" s="4">
+        <v>0</v>
+      </c>
+      <c r="CI55" s="4">
+        <v>0</v>
+      </c>
+      <c r="CJ55" s="4">
+        <v>0</v>
+      </c>
+      <c r="CK55" s="4">
+        <v>28</v>
+      </c>
+      <c r="CL55" s="4">
+        <v>0</v>
+      </c>
+      <c r="CM55" s="4">
+        <v>3</v>
+      </c>
+      <c r="CN55" s="4">
+        <v>0</v>
+      </c>
+      <c r="CO55" s="4">
+        <v>7</v>
+      </c>
+      <c r="CP55" s="4">
+        <v>11</v>
+      </c>
+      <c r="CQ55" s="4">
+        <v>9</v>
+      </c>
+      <c r="CR55" s="4">
+        <v>5</v>
+      </c>
+      <c r="CS55" s="4">
+        <v>39</v>
+      </c>
+      <c r="CT55" s="4">
+        <v>81</v>
+      </c>
+      <c r="CU55" s="4">
+        <v>318</v>
+      </c>
+      <c r="CV55" s="4">
+        <v>395</v>
+      </c>
+      <c r="CW55" s="4">
+        <v>103</v>
+      </c>
+      <c r="CX55" s="4">
+        <v>186</v>
+      </c>
+      <c r="CY55" s="4">
+        <v>29</v>
+      </c>
+      <c r="CZ55" s="4">
+        <v>90</v>
+      </c>
+      <c r="DA55" s="4">
+        <v>58</v>
+      </c>
+      <c r="DB55" s="4">
+        <v>73</v>
+      </c>
+      <c r="DC55" s="4">
+        <v>12</v>
+      </c>
+      <c r="DD55" s="4">
+        <v>35</v>
+      </c>
+      <c r="DE55" s="4">
+        <v>21</v>
+      </c>
+      <c r="DF55" s="4">
+        <v>6</v>
+      </c>
+      <c r="DG55" s="4">
+        <v>22</v>
+      </c>
+      <c r="DH55" s="4">
+        <v>2</v>
+      </c>
+      <c r="DI55" s="4">
+        <v>9</v>
+      </c>
+      <c r="DJ55" s="4">
+        <v>190</v>
+      </c>
+      <c r="DK55" s="4">
+        <v>47</v>
+      </c>
+      <c r="DL55" s="4">
+        <v>8</v>
+      </c>
+      <c r="DM55" s="4">
+        <v>0</v>
+      </c>
+      <c r="DN55" s="4">
+        <v>22</v>
+      </c>
+      <c r="DO55" s="4">
+        <v>8</v>
+      </c>
+      <c r="DP55" s="4">
+        <v>14</v>
+      </c>
+      <c r="DQ55" s="4">
+        <v>23</v>
+      </c>
+      <c r="DR55" s="4">
+        <v>30</v>
+      </c>
+      <c r="DS55" s="4">
+        <v>0</v>
+      </c>
+      <c r="DT55" s="4">
+        <v>0</v>
+      </c>
+      <c r="DU55" s="4">
+        <v>1</v>
+      </c>
+      <c r="DV55" s="4">
+        <v>2</v>
+      </c>
+      <c r="DW55" s="4">
+        <v>0</v>
+      </c>
+      <c r="DX55" s="4">
+        <v>0</v>
+      </c>
+      <c r="DY55" s="4">
+        <v>0</v>
+      </c>
+      <c r="DZ55" s="4">
+        <v>2</v>
+      </c>
+      <c r="EA55" s="4">
+        <v>1</v>
+      </c>
+      <c r="EB55" s="4">
+        <v>1</v>
+      </c>
+      <c r="EC55" s="4">
+        <v>2</v>
+      </c>
+      <c r="ED55" s="4">
+        <v>2</v>
+      </c>
+      <c r="EE55" s="4">
+        <v>0</v>
+      </c>
+      <c r="EF55" s="4">
+        <v>10</v>
+      </c>
+      <c r="EG55" s="4">
+        <v>1</v>
+      </c>
+      <c r="EH55" s="4">
+        <v>2</v>
+      </c>
+      <c r="EI55" s="7"/>
+      <c r="EJ55" s="7"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
+      <c r="A56" s="4">
+        <v>55</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="E56" s="4">
+        <v>1</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="G56" s="4">
+        <v>0</v>
+      </c>
+      <c r="H56" s="4">
+        <v>3</v>
+      </c>
+      <c r="I56" s="4">
+        <v>0</v>
+      </c>
+      <c r="J56" s="4">
+        <v>0</v>
+      </c>
+      <c r="K56" s="4">
+        <v>10</v>
+      </c>
+      <c r="L56" s="4">
+        <v>1</v>
+      </c>
+      <c r="M56" s="4">
+        <v>5</v>
+      </c>
+      <c r="N56" s="4">
+        <v>4</v>
+      </c>
+      <c r="O56" s="4">
+        <v>0</v>
+      </c>
+      <c r="P56" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="4">
+        <v>0</v>
+      </c>
+      <c r="R56" s="4">
+        <v>1</v>
+      </c>
+      <c r="S56" s="4">
+        <v>1</v>
+      </c>
+      <c r="T56" s="4">
+        <v>0</v>
+      </c>
+      <c r="U56" s="4">
+        <v>0</v>
+      </c>
+      <c r="V56" s="4">
+        <v>0</v>
+      </c>
+      <c r="W56" s="4">
+        <v>0</v>
+      </c>
+      <c r="X56" s="4">
+        <v>35</v>
+      </c>
+      <c r="Y56" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z56" s="4">
+        <v>4</v>
+      </c>
+      <c r="AA56" s="4">
+        <v>5</v>
+      </c>
+      <c r="AB56" s="4">
+        <v>4</v>
+      </c>
+      <c r="AC56" s="4">
+        <v>5</v>
+      </c>
+      <c r="AD56" s="4">
+        <v>2</v>
+      </c>
+      <c r="AE56" s="4">
+        <v>3</v>
+      </c>
+      <c r="AF56" s="4">
+        <v>40</v>
+      </c>
+      <c r="AG56" s="4">
+        <v>75</v>
+      </c>
+      <c r="AH56" s="4">
+        <v>191</v>
+      </c>
+      <c r="AI56" s="4">
+        <v>253</v>
+      </c>
+      <c r="AJ56" s="4">
+        <v>62</v>
+      </c>
+      <c r="AK56" s="4">
+        <v>103</v>
+      </c>
+      <c r="AL56" s="4">
+        <v>26</v>
+      </c>
+      <c r="AM56" s="4">
+        <v>39</v>
+      </c>
+      <c r="AN56" s="4">
+        <v>43</v>
+      </c>
+      <c r="AO56" s="4">
+        <v>45</v>
+      </c>
+      <c r="AP56" s="4">
+        <v>12</v>
+      </c>
+      <c r="AQ56" s="4">
+        <v>20</v>
+      </c>
+      <c r="AR56" s="4">
+        <v>11</v>
+      </c>
+      <c r="AS56" s="4">
+        <v>6</v>
+      </c>
+      <c r="AT56" s="4">
+        <v>24</v>
+      </c>
+      <c r="AU56" s="4">
+        <v>4</v>
+      </c>
+      <c r="AV56" s="4">
+        <v>17</v>
+      </c>
+      <c r="AW56" s="4">
+        <v>188</v>
+      </c>
+      <c r="AX56" s="4">
+        <v>36</v>
+      </c>
+      <c r="AY56" s="4">
+        <v>4</v>
+      </c>
+      <c r="AZ56" s="4">
+        <v>1</v>
+      </c>
+      <c r="BA56" s="4">
+        <v>22</v>
+      </c>
+      <c r="BB56" s="4">
+        <v>7</v>
+      </c>
+      <c r="BC56" s="4">
+        <v>15</v>
+      </c>
+      <c r="BD56" s="4">
+        <v>17</v>
+      </c>
+      <c r="BE56" s="4">
+        <v>29</v>
+      </c>
+      <c r="BF56" s="4">
+        <v>3</v>
+      </c>
+      <c r="BG56" s="4">
+        <v>0</v>
+      </c>
+      <c r="BH56" s="4">
+        <v>0</v>
+      </c>
+      <c r="BI56" s="4">
+        <v>5</v>
+      </c>
+      <c r="BJ56" s="4">
+        <v>0</v>
+      </c>
+      <c r="BK56" s="4">
+        <v>0</v>
+      </c>
+      <c r="BL56" s="4">
+        <v>0</v>
+      </c>
+      <c r="BM56" s="4">
+        <v>0</v>
+      </c>
+      <c r="BN56" s="4">
+        <v>0</v>
+      </c>
+      <c r="BO56" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP56" s="4">
+        <v>1</v>
+      </c>
+      <c r="BQ56" s="4">
+        <v>3</v>
+      </c>
+      <c r="BR56" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS56" s="4">
+        <v>24</v>
+      </c>
+      <c r="BT56" s="4">
+        <v>4</v>
+      </c>
+      <c r="BU56" s="4">
+        <v>11</v>
+      </c>
+      <c r="BV56" s="4">
+        <v>3</v>
+      </c>
+      <c r="BW56" s="4">
+        <v>0</v>
+      </c>
+      <c r="BX56" s="4">
+        <v>13</v>
+      </c>
+      <c r="BY56" s="4">
+        <v>7</v>
+      </c>
+      <c r="BZ56" s="4">
+        <v>2</v>
+      </c>
+      <c r="CA56" s="4">
+        <v>4</v>
+      </c>
+      <c r="CB56" s="4">
+        <v>0</v>
+      </c>
+      <c r="CC56" s="4">
+        <v>0</v>
+      </c>
+      <c r="CD56" s="4">
+        <v>0</v>
+      </c>
+      <c r="CE56" s="4">
+        <v>1</v>
+      </c>
+      <c r="CF56" s="4">
+        <v>1</v>
+      </c>
+      <c r="CG56" s="4">
+        <v>2</v>
+      </c>
+      <c r="CH56" s="4">
+        <v>1</v>
+      </c>
+      <c r="CI56" s="4">
+        <v>0</v>
+      </c>
+      <c r="CJ56" s="4">
+        <v>0</v>
+      </c>
+      <c r="CK56" s="4">
+        <v>42</v>
+      </c>
+      <c r="CL56" s="4">
+        <v>0</v>
+      </c>
+      <c r="CM56" s="4">
+        <v>7</v>
+      </c>
+      <c r="CN56" s="4">
+        <v>0</v>
+      </c>
+      <c r="CO56" s="4">
+        <v>11</v>
+      </c>
+      <c r="CP56" s="4">
+        <v>5</v>
+      </c>
+      <c r="CQ56" s="4">
+        <v>7</v>
+      </c>
+      <c r="CR56" s="4">
+        <v>5</v>
+      </c>
+      <c r="CS56" s="4">
+        <v>60</v>
+      </c>
+      <c r="CT56" s="4">
+        <v>80</v>
+      </c>
+      <c r="CU56" s="4">
+        <v>275</v>
+      </c>
+      <c r="CV56" s="4">
+        <v>342</v>
+      </c>
+      <c r="CW56" s="4">
+        <v>72</v>
+      </c>
+      <c r="CX56" s="4">
+        <v>179</v>
+      </c>
+      <c r="CY56" s="4">
+        <v>24</v>
+      </c>
+      <c r="CZ56" s="4">
+        <v>50</v>
+      </c>
+      <c r="DA56" s="4">
+        <v>78</v>
+      </c>
+      <c r="DB56" s="4">
+        <v>69</v>
+      </c>
+      <c r="DC56" s="4">
+        <v>28</v>
+      </c>
+      <c r="DD56" s="4">
+        <v>29</v>
+      </c>
+      <c r="DE56" s="4">
+        <v>24</v>
+      </c>
+      <c r="DF56" s="4">
+        <v>11</v>
+      </c>
+      <c r="DG56" s="4">
+        <v>16</v>
+      </c>
+      <c r="DH56" s="4">
+        <v>3</v>
+      </c>
+      <c r="DI56" s="4">
+        <v>19</v>
+      </c>
+      <c r="DJ56" s="4">
+        <v>200</v>
+      </c>
+      <c r="DK56" s="4">
+        <v>33</v>
+      </c>
+      <c r="DL56" s="4">
+        <v>4</v>
+      </c>
+      <c r="DM56" s="4">
+        <v>0</v>
+      </c>
+      <c r="DN56" s="4">
+        <v>9</v>
+      </c>
+      <c r="DO56" s="4">
+        <v>1</v>
+      </c>
+      <c r="DP56" s="4">
+        <v>8</v>
+      </c>
+      <c r="DQ56" s="4">
+        <v>13</v>
+      </c>
+      <c r="DR56" s="4">
+        <v>21</v>
+      </c>
+      <c r="DS56" s="4">
+        <v>0</v>
+      </c>
+      <c r="DT56" s="4">
+        <v>0</v>
+      </c>
+      <c r="DU56" s="4">
+        <v>1</v>
+      </c>
+      <c r="DV56" s="4">
+        <v>1</v>
+      </c>
+      <c r="DW56" s="4">
+        <v>0</v>
+      </c>
+      <c r="DX56" s="4">
+        <v>0</v>
+      </c>
+      <c r="DY56" s="4">
+        <v>0</v>
+      </c>
+      <c r="DZ56" s="4">
+        <v>1</v>
+      </c>
+      <c r="EA56" s="4">
+        <v>1</v>
+      </c>
+      <c r="EB56" s="4">
+        <v>0</v>
+      </c>
+      <c r="EC56" s="4">
+        <v>0</v>
+      </c>
+      <c r="ED56" s="4">
+        <v>4</v>
+      </c>
+      <c r="EE56" s="4">
+        <v>0</v>
+      </c>
+      <c r="EF56" s="4">
+        <v>12</v>
+      </c>
+      <c r="EG56" s="4">
+        <v>3</v>
+      </c>
+      <c r="EH56" s="4">
+        <v>6</v>
+      </c>
+      <c r="EI56" s="7"/>
+      <c r="EJ56" s="7"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
+      <c r="A57" s="4">
+        <v>56</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E57" s="4">
+        <v>1</v>
+      </c>
+      <c r="F57" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="G57" s="4">
+        <v>1</v>
+      </c>
+      <c r="H57" s="4">
+        <v>2</v>
+      </c>
+      <c r="I57" s="4">
+        <v>1</v>
+      </c>
+      <c r="J57" s="4">
+        <v>0</v>
+      </c>
+      <c r="K57" s="4">
+        <v>25</v>
+      </c>
+      <c r="L57" s="4">
+        <v>9</v>
+      </c>
+      <c r="M57" s="4">
+        <v>11</v>
+      </c>
+      <c r="N57" s="4">
+        <v>5</v>
+      </c>
+      <c r="O57" s="4">
+        <v>0</v>
+      </c>
+      <c r="P57" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q57" s="4">
+        <v>0</v>
+      </c>
+      <c r="R57" s="4">
+        <v>4</v>
+      </c>
+      <c r="S57" s="4">
+        <v>5</v>
+      </c>
+      <c r="T57" s="4">
+        <v>1</v>
+      </c>
+      <c r="U57" s="4">
+        <v>0</v>
+      </c>
+      <c r="V57" s="4">
+        <v>0</v>
+      </c>
+      <c r="W57" s="4">
+        <v>0</v>
+      </c>
+      <c r="X57" s="4">
+        <v>76</v>
+      </c>
+      <c r="Y57" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z57" s="4">
+        <v>9</v>
+      </c>
+      <c r="AA57" s="4">
+        <v>3</v>
+      </c>
+      <c r="AB57" s="4">
+        <v>15</v>
+      </c>
+      <c r="AC57" s="4">
+        <v>26</v>
+      </c>
+      <c r="AD57" s="4">
+        <v>26</v>
+      </c>
+      <c r="AE57" s="4">
+        <v>10</v>
+      </c>
+      <c r="AF57" s="4">
+        <v>64</v>
+      </c>
+      <c r="AG57" s="4">
+        <v>94</v>
+      </c>
+      <c r="AH57" s="4">
+        <v>670</v>
+      </c>
+      <c r="AI57" s="4">
+        <v>716</v>
+      </c>
+      <c r="AJ57" s="4">
+        <v>106</v>
+      </c>
+      <c r="AK57" s="4">
+        <v>512</v>
+      </c>
+      <c r="AL57" s="4">
+        <v>52</v>
+      </c>
+      <c r="AM57" s="4">
+        <v>132</v>
+      </c>
+      <c r="AN57" s="4">
+        <v>201</v>
+      </c>
+      <c r="AO57" s="4">
+        <v>203</v>
+      </c>
+      <c r="AP57" s="4">
+        <v>12</v>
+      </c>
+      <c r="AQ57" s="4">
+        <v>66</v>
+      </c>
+      <c r="AR57" s="4">
+        <v>65</v>
+      </c>
+      <c r="AS57" s="4">
+        <v>14</v>
+      </c>
+      <c r="AT57" s="4">
+        <v>25</v>
+      </c>
+      <c r="AU57" s="4">
+        <v>9</v>
+      </c>
+      <c r="AV57" s="4">
+        <v>36</v>
+      </c>
+      <c r="AW57" s="4">
+        <v>179</v>
+      </c>
+      <c r="AX57" s="4">
+        <v>38</v>
+      </c>
+      <c r="AY57" s="4">
+        <v>1</v>
+      </c>
+      <c r="AZ57" s="4">
+        <v>0</v>
+      </c>
+      <c r="BA57" s="4">
+        <v>13</v>
+      </c>
+      <c r="BB57" s="4">
+        <v>7</v>
+      </c>
+      <c r="BC57" s="4">
+        <v>6</v>
+      </c>
+      <c r="BD57" s="4">
+        <v>5</v>
+      </c>
+      <c r="BE57" s="4">
+        <v>7</v>
+      </c>
+      <c r="BF57" s="4">
+        <v>2</v>
+      </c>
+      <c r="BG57" s="4">
+        <v>0</v>
+      </c>
+      <c r="BH57" s="4">
+        <v>0</v>
+      </c>
+      <c r="BI57" s="4">
+        <v>3</v>
+      </c>
+      <c r="BJ57" s="4">
+        <v>0</v>
+      </c>
+      <c r="BK57" s="4">
+        <v>0</v>
+      </c>
+      <c r="BL57" s="4">
+        <v>0</v>
+      </c>
+      <c r="BM57" s="4">
+        <v>1</v>
+      </c>
+      <c r="BN57" s="4">
+        <v>1</v>
+      </c>
+      <c r="BO57" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP57" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ57" s="4">
+        <v>1</v>
+      </c>
+      <c r="BR57" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS57" s="4">
+        <v>7</v>
+      </c>
+      <c r="BT57" s="4">
+        <v>1</v>
+      </c>
+      <c r="BU57" s="4">
+        <v>2</v>
+      </c>
+      <c r="BV57" s="4">
+        <v>2</v>
+      </c>
+      <c r="BW57" s="4">
+        <v>0</v>
+      </c>
+      <c r="BX57" s="4">
+        <v>9</v>
+      </c>
+      <c r="BY57" s="4">
+        <v>5</v>
+      </c>
+      <c r="BZ57" s="4">
+        <v>3</v>
+      </c>
+      <c r="CA57" s="4">
+        <v>1</v>
+      </c>
+      <c r="CB57" s="4">
+        <v>1</v>
+      </c>
+      <c r="CC57" s="4">
+        <v>0</v>
+      </c>
+      <c r="CD57" s="4">
+        <v>1</v>
+      </c>
+      <c r="CE57" s="4">
+        <v>0</v>
+      </c>
+      <c r="CF57" s="4">
+        <v>2</v>
+      </c>
+      <c r="CG57" s="4">
+        <v>1</v>
+      </c>
+      <c r="CH57" s="4">
+        <v>0</v>
+      </c>
+      <c r="CI57" s="4">
+        <v>0</v>
+      </c>
+      <c r="CJ57" s="4">
+        <v>0</v>
+      </c>
+      <c r="CK57" s="4">
+        <v>27</v>
+      </c>
+      <c r="CL57" s="4">
+        <v>0</v>
+      </c>
+      <c r="CM57" s="4">
+        <v>1</v>
+      </c>
+      <c r="CN57" s="4">
+        <v>3</v>
+      </c>
+      <c r="CO57" s="4">
+        <v>14</v>
+      </c>
+      <c r="CP57" s="4">
+        <v>6</v>
+      </c>
+      <c r="CQ57" s="4">
+        <v>7</v>
+      </c>
+      <c r="CR57" s="4">
+        <v>3</v>
+      </c>
+      <c r="CS57" s="4">
+        <v>36</v>
+      </c>
+      <c r="CT57" s="4">
+        <v>80</v>
+      </c>
+      <c r="CU57" s="4">
+        <v>246</v>
+      </c>
+      <c r="CV57" s="4">
+        <v>309</v>
+      </c>
+      <c r="CW57" s="4">
+        <v>46</v>
+      </c>
+      <c r="CX57" s="4">
+        <v>173</v>
+      </c>
+      <c r="CY57" s="4">
+        <v>27</v>
+      </c>
+      <c r="CZ57" s="4">
+        <v>51</v>
+      </c>
+      <c r="DA57" s="4">
+        <v>71</v>
+      </c>
+      <c r="DB57" s="4">
+        <v>60</v>
+      </c>
+      <c r="DC57" s="4">
+        <v>10</v>
+      </c>
+      <c r="DD57" s="4">
+        <v>27</v>
+      </c>
+      <c r="DE57" s="4">
+        <v>21</v>
+      </c>
+      <c r="DF57" s="4">
+        <v>6</v>
+      </c>
+      <c r="DG57" s="4">
+        <v>0</v>
+      </c>
+      <c r="DH57" s="4">
+        <v>0</v>
+      </c>
+      <c r="DI57" s="4">
+        <v>1</v>
+      </c>
+      <c r="DJ57" s="4">
+        <v>177</v>
+      </c>
+      <c r="DK57" s="4">
+        <v>43</v>
+      </c>
+      <c r="DL57" s="4">
+        <v>5</v>
+      </c>
+      <c r="DM57" s="4">
+        <v>0</v>
+      </c>
+      <c r="DN57" s="4">
+        <v>20</v>
+      </c>
+      <c r="DO57" s="4">
+        <v>13</v>
+      </c>
+      <c r="DP57" s="4">
+        <v>7</v>
+      </c>
+      <c r="DQ57" s="4">
+        <v>21</v>
+      </c>
+      <c r="DR57" s="4">
+        <v>29</v>
+      </c>
+      <c r="DS57" s="4">
+        <v>1</v>
+      </c>
+      <c r="DT57" s="4">
+        <v>0</v>
+      </c>
+      <c r="DU57" s="4">
+        <v>0</v>
+      </c>
+      <c r="DV57" s="4">
+        <v>8</v>
+      </c>
+      <c r="DW57" s="4">
+        <v>0</v>
+      </c>
+      <c r="DX57" s="4">
+        <v>0</v>
+      </c>
+      <c r="DY57" s="4">
+        <v>0</v>
+      </c>
+      <c r="DZ57" s="4">
+        <v>4</v>
+      </c>
+      <c r="EA57" s="4">
+        <v>2</v>
+      </c>
+      <c r="EB57" s="4">
+        <v>2</v>
+      </c>
+      <c r="EC57" s="4">
+        <v>0</v>
+      </c>
+      <c r="ED57" s="4">
+        <v>3</v>
+      </c>
+      <c r="EE57" s="4">
+        <v>1</v>
+      </c>
+      <c r="EF57" s="4">
+        <v>9</v>
+      </c>
+      <c r="EG57" s="4">
+        <v>1</v>
+      </c>
+      <c r="EH57" s="4">
+        <v>1</v>
+      </c>
+      <c r="EI57" s="7"/>
+      <c r="EJ57" s="7"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
+      <c r="A58" s="4">
+        <v>57</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="E58" s="4">
+        <v>1</v>
+      </c>
+      <c r="F58" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="G58" s="4">
+        <v>1</v>
+      </c>
+      <c r="H58" s="4">
+        <v>0</v>
+      </c>
+      <c r="I58" s="4">
+        <v>1</v>
+      </c>
+      <c r="J58" s="4">
+        <v>0</v>
+      </c>
+      <c r="K58" s="4">
+        <v>17</v>
+      </c>
+      <c r="L58" s="4">
+        <v>9</v>
+      </c>
+      <c r="M58" s="4">
+        <v>3</v>
+      </c>
+      <c r="N58" s="4">
+        <v>5</v>
+      </c>
+      <c r="O58" s="4">
+        <v>0</v>
+      </c>
+      <c r="P58" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="4">
+        <v>0</v>
+      </c>
+      <c r="R58" s="4">
+        <v>4</v>
+      </c>
+      <c r="S58" s="4">
+        <v>1</v>
+      </c>
+      <c r="T58" s="4">
+        <v>1</v>
+      </c>
+      <c r="U58" s="4">
+        <v>0</v>
+      </c>
+      <c r="V58" s="4">
+        <v>0</v>
+      </c>
+      <c r="W58" s="4">
+        <v>0</v>
+      </c>
+      <c r="X58" s="4">
+        <v>41</v>
+      </c>
+      <c r="Y58" s="4">
+        <v>2</v>
+      </c>
+      <c r="Z58" s="4">
+        <v>4</v>
+      </c>
+      <c r="AA58" s="4">
+        <v>2</v>
+      </c>
+      <c r="AB58" s="4">
+        <v>29</v>
+      </c>
+      <c r="AC58" s="4">
+        <v>12</v>
+      </c>
+      <c r="AD58" s="4">
+        <v>13</v>
+      </c>
+      <c r="AE58" s="4">
+        <v>7</v>
+      </c>
+      <c r="AF58" s="4">
+        <v>41</v>
+      </c>
+      <c r="AG58" s="4">
+        <v>80</v>
+      </c>
+      <c r="AH58" s="4">
+        <v>270</v>
+      </c>
+      <c r="AI58" s="4">
+        <v>339</v>
+      </c>
+      <c r="AJ58" s="4">
+        <v>95</v>
+      </c>
+      <c r="AK58" s="4">
+        <v>154</v>
+      </c>
+      <c r="AL58" s="4">
+        <v>21</v>
+      </c>
+      <c r="AM58" s="4">
+        <v>60</v>
+      </c>
+      <c r="AN58" s="4">
+        <v>55</v>
+      </c>
+      <c r="AO58" s="4">
+        <v>66</v>
+      </c>
+      <c r="AP58" s="4">
+        <v>11</v>
+      </c>
+      <c r="AQ58" s="4">
+        <v>28</v>
+      </c>
+      <c r="AR58" s="4">
+        <v>23</v>
+      </c>
+      <c r="AS58" s="4">
+        <v>12</v>
+      </c>
+      <c r="AT58" s="4">
+        <v>40</v>
+      </c>
+      <c r="AU58" s="4">
+        <v>4</v>
+      </c>
+      <c r="AV58" s="4">
+        <v>10</v>
+      </c>
+      <c r="AW58" s="4">
+        <v>178</v>
+      </c>
+      <c r="AX58" s="4">
+        <v>43</v>
+      </c>
+      <c r="AY58" s="4">
+        <v>2</v>
+      </c>
+      <c r="AZ58" s="4">
+        <v>0</v>
+      </c>
+      <c r="BA58" s="4">
+        <v>18</v>
+      </c>
+      <c r="BB58" s="4">
+        <v>5</v>
+      </c>
+      <c r="BC58" s="4">
+        <v>13</v>
+      </c>
+      <c r="BD58" s="4">
+        <v>9</v>
+      </c>
+      <c r="BE58" s="4">
+        <v>10</v>
+      </c>
+      <c r="BF58" s="4">
+        <v>0</v>
+      </c>
+      <c r="BG58" s="4">
+        <v>0</v>
+      </c>
+      <c r="BH58" s="4">
+        <v>1</v>
+      </c>
+      <c r="BI58" s="4">
+        <v>2</v>
+      </c>
+      <c r="BJ58" s="4">
+        <v>0</v>
+      </c>
+      <c r="BK58" s="4">
+        <v>0</v>
+      </c>
+      <c r="BL58" s="4">
+        <v>0</v>
+      </c>
+      <c r="BM58" s="4">
+        <v>1</v>
+      </c>
+      <c r="BN58" s="4">
+        <v>0</v>
+      </c>
+      <c r="BO58" s="4">
+        <v>1</v>
+      </c>
+      <c r="BP58" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ58" s="4">
+        <v>1</v>
+      </c>
+      <c r="BR58" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS58" s="4">
+        <v>16</v>
+      </c>
+      <c r="BT58" s="4">
+        <v>1</v>
+      </c>
+      <c r="BU58" s="4">
+        <v>3</v>
+      </c>
+      <c r="BV58" s="4">
+        <v>0</v>
+      </c>
+      <c r="BW58" s="4">
+        <v>0</v>
+      </c>
+      <c r="BX58" s="4">
+        <v>8</v>
+      </c>
+      <c r="BY58" s="4">
+        <v>2</v>
+      </c>
+      <c r="BZ58" s="4">
+        <v>4</v>
+      </c>
+      <c r="CA58" s="4">
+        <v>2</v>
+      </c>
+      <c r="CB58" s="4">
+        <v>0</v>
+      </c>
+      <c r="CC58" s="4">
+        <v>0</v>
+      </c>
+      <c r="CD58" s="4">
+        <v>0</v>
+      </c>
+      <c r="CE58" s="4">
+        <v>1</v>
+      </c>
+      <c r="CF58" s="4">
+        <v>2</v>
+      </c>
+      <c r="CG58" s="4">
+        <v>0</v>
+      </c>
+      <c r="CH58" s="4">
+        <v>0</v>
+      </c>
+      <c r="CI58" s="4">
+        <v>0</v>
+      </c>
+      <c r="CJ58" s="4">
+        <v>0</v>
+      </c>
+      <c r="CK58" s="4">
+        <v>48</v>
+      </c>
+      <c r="CL58" s="4">
+        <v>0</v>
+      </c>
+      <c r="CM58" s="4">
+        <v>2</v>
+      </c>
+      <c r="CN58" s="4">
+        <v>0</v>
+      </c>
+      <c r="CO58" s="4">
+        <v>26</v>
+      </c>
+      <c r="CP58" s="4">
+        <v>17</v>
+      </c>
+      <c r="CQ58" s="4">
+        <v>11</v>
+      </c>
+      <c r="CR58" s="4">
+        <v>10</v>
+      </c>
+      <c r="CS58" s="4">
+        <v>59</v>
+      </c>
+      <c r="CT58" s="4">
+        <v>88</v>
+      </c>
+      <c r="CU58" s="4">
+        <v>467</v>
+      </c>
+      <c r="CV58" s="4">
+        <v>533</v>
+      </c>
+      <c r="CW58" s="4">
+        <v>135</v>
+      </c>
+      <c r="CX58" s="4">
+        <v>304</v>
+      </c>
+      <c r="CY58" s="4">
+        <v>28</v>
+      </c>
+      <c r="CZ58" s="4">
+        <v>93</v>
+      </c>
+      <c r="DA58" s="4">
+        <v>118</v>
+      </c>
+      <c r="DB58" s="4">
+        <v>121</v>
+      </c>
+      <c r="DC58" s="4">
+        <v>18</v>
+      </c>
+      <c r="DD58" s="4">
+        <v>44</v>
+      </c>
+      <c r="DE58" s="4">
+        <v>41</v>
+      </c>
+      <c r="DF58" s="4">
+        <v>6</v>
+      </c>
+      <c r="DG58" s="4">
+        <v>0</v>
+      </c>
+      <c r="DH58" s="4">
+        <v>0</v>
+      </c>
+      <c r="DI58" s="4">
+        <v>9</v>
+      </c>
+      <c r="DJ58" s="4">
+        <v>185</v>
+      </c>
+      <c r="DK58" s="4">
+        <v>34</v>
+      </c>
+      <c r="DL58" s="4">
+        <v>5</v>
+      </c>
+      <c r="DM58" s="4">
+        <v>0</v>
+      </c>
+      <c r="DN58" s="4">
+        <v>33</v>
+      </c>
+      <c r="DO58" s="4">
+        <v>13</v>
+      </c>
+      <c r="DP58" s="4">
+        <v>20</v>
+      </c>
+      <c r="DQ58" s="4">
+        <v>20</v>
+      </c>
+      <c r="DR58" s="4">
+        <v>27</v>
+      </c>
+      <c r="DS58" s="4">
+        <v>1</v>
+      </c>
+      <c r="DT58" s="4">
+        <v>0</v>
+      </c>
+      <c r="DU58" s="4">
+        <v>0</v>
+      </c>
+      <c r="DV58" s="4">
+        <v>8</v>
+      </c>
+      <c r="DW58" s="4">
+        <v>1</v>
+      </c>
+      <c r="DX58" s="4">
+        <v>0</v>
+      </c>
+      <c r="DY58" s="4">
+        <v>0</v>
+      </c>
+      <c r="DZ58" s="4">
+        <v>4</v>
+      </c>
+      <c r="EA58" s="4">
+        <v>1</v>
+      </c>
+      <c r="EB58" s="4">
+        <v>3</v>
+      </c>
+      <c r="EC58" s="4">
+        <v>0</v>
+      </c>
+      <c r="ED58" s="4">
+        <v>5</v>
+      </c>
+      <c r="EE58" s="4">
+        <v>0</v>
+      </c>
+      <c r="EF58" s="4">
+        <v>11</v>
+      </c>
+      <c r="EG58" s="4">
+        <v>5</v>
+      </c>
+      <c r="EH58" s="4">
+        <v>8</v>
+      </c>
+      <c r="EI58" s="7"/>
+      <c r="EJ58" s="7"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
+      <c r="A59" s="4">
+        <v>58</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="E59" s="4">
+        <v>1</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="G59" s="4">
+        <v>3</v>
+      </c>
+      <c r="H59" s="4">
+        <v>1</v>
+      </c>
+      <c r="I59" s="4">
+        <v>3</v>
+      </c>
+      <c r="J59" s="4">
+        <v>0</v>
+      </c>
+      <c r="K59" s="4">
+        <v>15</v>
+      </c>
+      <c r="L59" s="4">
+        <v>6</v>
+      </c>
+      <c r="M59" s="4">
+        <v>5</v>
+      </c>
+      <c r="N59" s="4">
+        <v>4</v>
+      </c>
+      <c r="O59" s="4">
+        <v>0</v>
+      </c>
+      <c r="P59" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="4">
+        <v>0</v>
+      </c>
+      <c r="R59" s="4">
+        <v>1</v>
+      </c>
+      <c r="S59" s="4">
+        <v>0</v>
+      </c>
+      <c r="T59" s="4">
+        <v>2</v>
+      </c>
+      <c r="U59" s="4">
+        <v>0</v>
+      </c>
+      <c r="V59" s="4">
+        <v>0</v>
+      </c>
+      <c r="W59" s="4">
+        <v>0</v>
+      </c>
+      <c r="X59" s="4">
+        <v>46</v>
+      </c>
+      <c r="Y59" s="4">
+        <v>1</v>
+      </c>
+      <c r="Z59" s="4">
+        <v>9</v>
+      </c>
+      <c r="AA59" s="4">
+        <v>1</v>
+      </c>
+      <c r="AB59" s="4">
+        <v>20</v>
+      </c>
+      <c r="AC59" s="4">
+        <v>13</v>
+      </c>
+      <c r="AD59" s="4">
+        <v>7</v>
+      </c>
+      <c r="AE59" s="4">
+        <v>3</v>
+      </c>
+      <c r="AF59" s="4">
+        <v>62</v>
+      </c>
+      <c r="AG59" s="4">
+        <v>91</v>
+      </c>
+      <c r="AH59" s="4">
+        <v>585</v>
+      </c>
+      <c r="AI59" s="4">
+        <v>643</v>
+      </c>
+      <c r="AJ59" s="4">
+        <v>122</v>
+      </c>
+      <c r="AK59" s="4">
+        <v>401</v>
+      </c>
+      <c r="AL59" s="4">
+        <v>62</v>
+      </c>
+      <c r="AM59" s="4">
+        <v>94</v>
+      </c>
+      <c r="AN59" s="4">
+        <v>169</v>
+      </c>
+      <c r="AO59" s="4">
+        <v>169</v>
+      </c>
+      <c r="AP59" s="4">
+        <v>13</v>
+      </c>
+      <c r="AQ59" s="4">
+        <v>64</v>
+      </c>
+      <c r="AR59" s="4">
+        <v>30</v>
+      </c>
+      <c r="AS59" s="4">
+        <v>18</v>
+      </c>
+      <c r="AT59" s="4">
+        <v>38</v>
+      </c>
+      <c r="AU59" s="4">
+        <v>10</v>
+      </c>
+      <c r="AV59" s="4">
+        <v>26</v>
+      </c>
+      <c r="AW59" s="4">
+        <v>153</v>
+      </c>
+      <c r="AX59" s="4">
+        <v>34</v>
+      </c>
+      <c r="AY59" s="4">
+        <v>1</v>
+      </c>
+      <c r="AZ59" s="4">
+        <v>0</v>
+      </c>
+      <c r="BA59" s="4">
+        <v>7</v>
+      </c>
+      <c r="BB59" s="4">
+        <v>2</v>
+      </c>
+      <c r="BC59" s="4">
+        <v>5</v>
+      </c>
+      <c r="BD59" s="4">
+        <v>14</v>
+      </c>
+      <c r="BE59" s="4">
+        <v>16</v>
+      </c>
+      <c r="BF59" s="4">
+        <v>1</v>
+      </c>
+      <c r="BG59" s="4">
+        <v>0</v>
+      </c>
+      <c r="BH59" s="4">
+        <v>0</v>
+      </c>
+      <c r="BI59" s="4">
+        <v>2</v>
+      </c>
+      <c r="BJ59" s="4">
+        <v>0</v>
+      </c>
+      <c r="BK59" s="4">
+        <v>0</v>
+      </c>
+      <c r="BL59" s="4">
+        <v>0</v>
+      </c>
+      <c r="BM59" s="4">
+        <v>4</v>
+      </c>
+      <c r="BN59" s="4">
+        <v>4</v>
+      </c>
+      <c r="BO59" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP59" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ59" s="4">
+        <v>1</v>
+      </c>
+      <c r="BR59" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS59" s="4">
+        <v>10</v>
+      </c>
+      <c r="BT59" s="4">
+        <v>2</v>
+      </c>
+      <c r="BU59" s="4">
+        <v>4</v>
+      </c>
+      <c r="BV59" s="4">
+        <v>1</v>
+      </c>
+      <c r="BW59" s="4">
+        <v>0</v>
+      </c>
+      <c r="BX59" s="4">
+        <v>8</v>
+      </c>
+      <c r="BY59" s="4">
+        <v>3</v>
+      </c>
+      <c r="BZ59" s="4">
+        <v>4</v>
+      </c>
+      <c r="CA59" s="4">
+        <v>1</v>
+      </c>
+      <c r="CB59" s="4">
+        <v>0</v>
+      </c>
+      <c r="CC59" s="4">
+        <v>0</v>
+      </c>
+      <c r="CD59" s="4">
+        <v>0</v>
+      </c>
+      <c r="CE59" s="4">
+        <v>0</v>
+      </c>
+      <c r="CF59" s="4">
+        <v>1</v>
+      </c>
+      <c r="CG59" s="4">
+        <v>1</v>
+      </c>
+      <c r="CH59" s="4">
+        <v>0</v>
+      </c>
+      <c r="CI59" s="4">
+        <v>0</v>
+      </c>
+      <c r="CJ59" s="4">
+        <v>0</v>
+      </c>
+      <c r="CK59" s="4">
+        <v>27</v>
+      </c>
+      <c r="CL59" s="4">
+        <v>0</v>
+      </c>
+      <c r="CM59" s="4">
+        <v>1</v>
+      </c>
+      <c r="CN59" s="4">
+        <v>1</v>
+      </c>
+      <c r="CO59" s="4">
+        <v>17</v>
+      </c>
+      <c r="CP59" s="4">
+        <v>4</v>
+      </c>
+      <c r="CQ59" s="4">
+        <v>4</v>
+      </c>
+      <c r="CR59" s="4">
+        <v>2</v>
+      </c>
+      <c r="CS59" s="4">
+        <v>38</v>
+      </c>
+      <c r="CT59" s="4">
+        <v>82</v>
+      </c>
+      <c r="CU59" s="4">
+        <v>267</v>
+      </c>
+      <c r="CV59" s="4">
+        <v>325</v>
+      </c>
+      <c r="CW59" s="4">
+        <v>78</v>
+      </c>
+      <c r="CX59" s="4">
+        <v>155</v>
+      </c>
+      <c r="CY59" s="4">
+        <v>34</v>
+      </c>
+      <c r="CZ59" s="4">
+        <v>47</v>
+      </c>
+      <c r="DA59" s="4">
+        <v>73</v>
+      </c>
+      <c r="DB59" s="4">
+        <v>70</v>
+      </c>
+      <c r="DC59" s="4">
+        <v>11</v>
+      </c>
+      <c r="DD59" s="4">
+        <v>23</v>
+      </c>
+      <c r="DE59" s="4">
+        <v>12</v>
+      </c>
+      <c r="DF59" s="4">
+        <v>7</v>
+      </c>
+      <c r="DG59" s="4">
+        <v>27</v>
+      </c>
+      <c r="DH59" s="4">
+        <v>3</v>
+      </c>
+      <c r="DI59" s="4">
+        <v>11</v>
+      </c>
+      <c r="DJ59" s="4">
+        <v>154</v>
+      </c>
+      <c r="DK59" s="4">
+        <v>37</v>
+      </c>
+      <c r="DL59" s="4">
+        <v>4</v>
+      </c>
+      <c r="DM59" s="4">
+        <v>0</v>
+      </c>
+      <c r="DN59" s="4">
+        <v>16</v>
+      </c>
+      <c r="DO59" s="4">
+        <v>6</v>
+      </c>
+      <c r="DP59" s="4">
+        <v>10</v>
+      </c>
+      <c r="DQ59" s="4">
+        <v>24</v>
+      </c>
+      <c r="DR59" s="4">
+        <v>24</v>
+      </c>
+      <c r="DS59" s="4">
+        <v>3</v>
+      </c>
+      <c r="DT59" s="4">
+        <v>0</v>
+      </c>
+      <c r="DU59" s="4">
+        <v>0</v>
+      </c>
+      <c r="DV59" s="4">
+        <v>3</v>
+      </c>
+      <c r="DW59" s="4">
+        <v>0</v>
+      </c>
+      <c r="DX59" s="4">
+        <v>0</v>
+      </c>
+      <c r="DY59" s="4">
+        <v>0</v>
+      </c>
+      <c r="DZ59" s="4">
+        <v>3</v>
+      </c>
+      <c r="EA59" s="4">
+        <v>2</v>
+      </c>
+      <c r="EB59" s="4">
+        <v>1</v>
+      </c>
+      <c r="EC59" s="4">
+        <v>1</v>
+      </c>
+      <c r="ED59" s="4">
+        <v>3</v>
+      </c>
+      <c r="EE59" s="4">
+        <v>0</v>
+      </c>
+      <c r="EF59" s="4">
+        <v>13</v>
+      </c>
+      <c r="EG59" s="4">
+        <v>4</v>
+      </c>
+      <c r="EH59" s="4">
+        <v>8</v>
+      </c>
+      <c r="EI59" s="7"/>
+      <c r="EJ59" s="7"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
+      <c r="A60" s="4">
+        <v>59</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="E60" s="4">
+        <v>1</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G60" s="4">
+        <v>1</v>
+      </c>
+      <c r="H60" s="4">
+        <v>1</v>
+      </c>
+      <c r="I60" s="4">
+        <v>1</v>
+      </c>
+      <c r="J60" s="4">
+        <v>0</v>
+      </c>
+      <c r="K60" s="4">
+        <v>18</v>
+      </c>
+      <c r="L60" s="4">
+        <v>9</v>
+      </c>
+      <c r="M60" s="4">
+        <v>5</v>
+      </c>
+      <c r="N60" s="4">
+        <v>4</v>
+      </c>
+      <c r="O60" s="4">
+        <v>0</v>
+      </c>
+      <c r="P60" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q60" s="4">
+        <v>0</v>
+      </c>
+      <c r="R60" s="4">
+        <v>4</v>
+      </c>
+      <c r="S60" s="4">
+        <v>4</v>
+      </c>
+      <c r="T60" s="4">
+        <v>1</v>
+      </c>
+      <c r="U60" s="4">
+        <v>0</v>
+      </c>
+      <c r="V60" s="4">
+        <v>0</v>
+      </c>
+      <c r="W60" s="4">
+        <v>0</v>
+      </c>
+      <c r="X60" s="4">
+        <v>58</v>
+      </c>
+      <c r="Y60" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z60" s="4">
+        <v>6</v>
+      </c>
+      <c r="AA60" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB60" s="4">
+        <v>9</v>
+      </c>
+      <c r="AC60" s="4">
+        <v>18</v>
+      </c>
+      <c r="AD60" s="4">
+        <v>16</v>
+      </c>
+      <c r="AE60" s="4">
+        <v>6</v>
+      </c>
+      <c r="AF60" s="4">
+        <v>47</v>
+      </c>
+      <c r="AG60" s="4">
+        <v>88</v>
+      </c>
+      <c r="AH60" s="4">
+        <v>453</v>
+      </c>
+      <c r="AI60" s="4">
+        <v>512</v>
+      </c>
+      <c r="AJ60" s="4">
+        <v>87</v>
+      </c>
+      <c r="AK60" s="4">
+        <v>328</v>
+      </c>
+      <c r="AL60" s="4">
+        <v>38</v>
+      </c>
+      <c r="AM60" s="4">
+        <v>83</v>
+      </c>
+      <c r="AN60" s="4">
+        <v>125</v>
+      </c>
+      <c r="AO60" s="4">
+        <v>117</v>
+      </c>
+      <c r="AP60" s="4">
+        <v>15</v>
+      </c>
+      <c r="AQ60" s="4">
+        <v>45</v>
+      </c>
+      <c r="AR60" s="4">
+        <v>43</v>
+      </c>
+      <c r="AS60" s="4">
+        <v>15</v>
+      </c>
+      <c r="AT60" s="4">
+        <v>35</v>
+      </c>
+      <c r="AU60" s="4">
+        <v>8</v>
+      </c>
+      <c r="AV60" s="4">
+        <v>23</v>
+      </c>
+      <c r="AW60" s="4">
+        <v>165</v>
+      </c>
+      <c r="AX60" s="4">
+        <v>43</v>
+      </c>
+      <c r="AY60" s="4">
+        <v>2</v>
+      </c>
+      <c r="AZ60" s="4">
+        <v>0</v>
+      </c>
+      <c r="BA60" s="4">
+        <v>22</v>
+      </c>
+      <c r="BB60" s="4">
+        <v>7</v>
+      </c>
+      <c r="BC60" s="4">
+        <v>15</v>
+      </c>
+      <c r="BD60" s="4">
+        <v>5</v>
+      </c>
+      <c r="BE60" s="4">
+        <v>6</v>
+      </c>
+      <c r="BF60" s="4">
+        <v>1</v>
+      </c>
+      <c r="BG60" s="4">
+        <v>0</v>
+      </c>
+      <c r="BH60" s="4">
+        <v>0</v>
+      </c>
+      <c r="BI60" s="4">
+        <v>1</v>
+      </c>
+      <c r="BJ60" s="4">
+        <v>0</v>
+      </c>
+      <c r="BK60" s="4">
+        <v>0</v>
+      </c>
+      <c r="BL60" s="4">
+        <v>0</v>
+      </c>
+      <c r="BM60" s="4">
+        <v>2</v>
+      </c>
+      <c r="BN60" s="4">
+        <v>0</v>
+      </c>
+      <c r="BO60" s="4">
+        <v>2</v>
+      </c>
+      <c r="BP60" s="4">
+        <v>1</v>
+      </c>
+      <c r="BQ60" s="4">
+        <v>2</v>
+      </c>
+      <c r="BR60" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS60" s="4">
+        <v>15</v>
+      </c>
+      <c r="BT60" s="4">
+        <v>2</v>
+      </c>
+      <c r="BU60" s="4">
+        <v>6</v>
+      </c>
+      <c r="BV60" s="4">
+        <v>1</v>
+      </c>
+      <c r="BW60" s="4">
+        <v>0</v>
+      </c>
+      <c r="BX60" s="4">
+        <v>5</v>
+      </c>
+      <c r="BY60" s="4">
+        <v>2</v>
+      </c>
+      <c r="BZ60" s="4">
+        <v>1</v>
+      </c>
+      <c r="CA60" s="4">
+        <v>2</v>
+      </c>
+      <c r="CB60" s="4">
+        <v>0</v>
+      </c>
+      <c r="CC60" s="4">
+        <v>0</v>
+      </c>
+      <c r="CD60" s="4">
+        <v>0</v>
+      </c>
+      <c r="CE60" s="4">
+        <v>0</v>
+      </c>
+      <c r="CF60" s="4">
+        <v>1</v>
+      </c>
+      <c r="CG60" s="4">
+        <v>1</v>
+      </c>
+      <c r="CH60" s="4">
+        <v>0</v>
+      </c>
+      <c r="CI60" s="4">
+        <v>0</v>
+      </c>
+      <c r="CJ60" s="4">
+        <v>0</v>
+      </c>
+      <c r="CK60" s="4">
+        <v>28</v>
+      </c>
+      <c r="CL60" s="4">
+        <v>0</v>
+      </c>
+      <c r="CM60" s="4">
+        <v>0</v>
+      </c>
+      <c r="CN60" s="4">
+        <v>1</v>
+      </c>
+      <c r="CO60" s="4">
+        <v>10</v>
+      </c>
+      <c r="CP60" s="4">
+        <v>12</v>
+      </c>
+      <c r="CQ60" s="4">
+        <v>10</v>
+      </c>
+      <c r="CR60" s="4">
+        <v>4</v>
+      </c>
+      <c r="CS60" s="4">
+        <v>53</v>
+      </c>
+      <c r="CT60" s="4">
+        <v>88</v>
+      </c>
+      <c r="CU60" s="4">
+        <v>472</v>
+      </c>
+      <c r="CV60" s="4">
+        <v>534</v>
+      </c>
+      <c r="CW60" s="4">
+        <v>97</v>
+      </c>
+      <c r="CX60" s="4">
+        <v>353</v>
+      </c>
+      <c r="CY60" s="4">
+        <v>22</v>
+      </c>
+      <c r="CZ60" s="4">
+        <v>85</v>
+      </c>
+      <c r="DA60" s="4">
+        <v>123</v>
+      </c>
+      <c r="DB60" s="4">
+        <v>125</v>
+      </c>
+      <c r="DC60" s="4">
+        <v>15</v>
+      </c>
+      <c r="DD60" s="4">
+        <v>41</v>
+      </c>
+      <c r="DE60" s="4">
+        <v>35</v>
+      </c>
+      <c r="DF60" s="4">
+        <v>4</v>
+      </c>
+      <c r="DG60" s="4">
+        <v>0</v>
+      </c>
+      <c r="DH60" s="4">
+        <v>0</v>
+      </c>
+      <c r="DI60" s="4">
+        <v>2</v>
+      </c>
+      <c r="DJ60" s="4">
+        <v>165</v>
+      </c>
+      <c r="DK60" s="4">
+        <v>26</v>
+      </c>
+      <c r="DL60" s="4">
+        <v>4</v>
+      </c>
+      <c r="DM60" s="4">
+        <v>0</v>
+      </c>
+      <c r="DN60" s="4">
+        <v>11</v>
+      </c>
+      <c r="DO60" s="4">
+        <v>5</v>
+      </c>
+      <c r="DP60" s="4">
+        <v>6</v>
+      </c>
+      <c r="DQ60" s="4">
+        <v>11</v>
+      </c>
+      <c r="DR60" s="4">
+        <v>19</v>
+      </c>
+      <c r="DS60" s="4">
+        <v>1</v>
+      </c>
+      <c r="DT60" s="4">
+        <v>0</v>
+      </c>
+      <c r="DU60" s="4">
+        <v>0</v>
+      </c>
+      <c r="DV60" s="4">
+        <v>8</v>
+      </c>
+      <c r="DW60" s="4">
+        <v>0</v>
+      </c>
+      <c r="DX60" s="4">
+        <v>0</v>
+      </c>
+      <c r="DY60" s="4">
+        <v>0</v>
+      </c>
+      <c r="DZ60" s="4">
+        <v>3</v>
+      </c>
+      <c r="EA60" s="4">
+        <v>1</v>
+      </c>
+      <c r="EB60" s="4">
+        <v>2</v>
+      </c>
+      <c r="EC60" s="4">
+        <v>0</v>
+      </c>
+      <c r="ED60" s="4">
+        <v>3</v>
+      </c>
+      <c r="EE60" s="4">
+        <v>0</v>
+      </c>
+      <c r="EF60" s="4">
+        <v>14</v>
+      </c>
+      <c r="EG60" s="4">
+        <v>3</v>
+      </c>
+      <c r="EH60" s="4">
+        <v>5</v>
+      </c>
+      <c r="EI60" s="7"/>
+      <c r="EJ60" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>